<commit_message>
Record verified docket status for 11 A-tier cases
Folds Register of Actions data into the tracker: 10 of 11 confirmed still
open, 1 closed by final discharge. Adds a Court Flagged Delinquent column
capturing Notices of Failure to Perform Duties and sanction OSCs, which
four of the eleven cases carry.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KmrMHojnrvSNV7tKWJ6vCj
</commit_message>
<xml_diff>
--- a/San_Diego_ATier_Verification_Tracker.xlsx
+++ b/San_Diego_ATier_Verification_Tracker.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Tally" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Verify'!$A$1:$S$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Verify'!$A$1:$T$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,8 +67,22 @@
       <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +97,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -112,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,17 +152,36 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -706,17 +754,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:T29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
@@ -763,65 +811,70 @@
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
+          <t>Court Flagged Delinquent</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Equity</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Decedent</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Property Address</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>Property Status</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="O1" s="5" t="inlineStr">
         <is>
           <t>Authority</t>
         </is>
       </c>
-      <c r="O1" s="5" t="inlineStr">
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>Petitioner</t>
         </is>
       </c>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>Pet. City/ST</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
         <is>
           <t>Attorney</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>Attorney Phone</t>
         </is>
       </c>
-      <c r="S1" s="5" t="inlineStr">
+      <c r="T1" s="5" t="inlineStr">
         <is>
           <t>Why It Scores</t>
         </is>
@@ -834,63 +887,64 @@
         </is>
       </c>
       <c r="B2" s="7" t="n"/>
-      <c r="C2" s="8" t="n"/>
+      <c r="C2" s="17" t="n"/>
       <c r="D2" s="7" t="n"/>
-      <c r="E2" s="8" t="n"/>
+      <c r="E2" s="17" t="n"/>
       <c r="F2" s="7" t="n"/>
-      <c r="G2" s="7" t="n"/>
-      <c r="H2" s="9" t="n">
+      <c r="G2" s="18" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="9" t="n">
         <v>73</v>
       </c>
-      <c r="I2" s="10" t="n">
+      <c r="J2" s="19" t="n">
         <v>1094112</v>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>Donna Lee Bura</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>8838 Hunter Pass</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="M2" s="6" t="inlineStr">
         <is>
           <t>Alpine</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="P2" s="6" t="inlineStr">
         <is>
           <t>Christopher J. Bura</t>
         </is>
       </c>
-      <c r="P2" s="6" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
         <is>
           <t>Springhill TN</t>
         </is>
       </c>
-      <c r="Q2" s="6" t="inlineStr">
+      <c r="R2" s="6" t="inlineStr">
         <is>
           <t>Julie K. Hardisty</t>
         </is>
       </c>
-      <c r="R2" s="6" t="inlineStr">
+      <c r="S2" s="6" t="inlineStr">
         <is>
           <t>925-689-9940</t>
         </is>
       </c>
-      <c r="S2" s="11" t="inlineStr">
+      <c r="T2" s="11" t="inlineStr">
         <is>
           <t>26mo old; $1M+ equity; vacant/absentee; limited authority (court confirmation); out-of-county heir</t>
         </is>
@@ -903,63 +957,64 @@
         </is>
       </c>
       <c r="B3" s="7" t="n"/>
-      <c r="C3" s="8" t="n"/>
+      <c r="C3" s="17" t="n"/>
       <c r="D3" s="7" t="n"/>
-      <c r="E3" s="8" t="n"/>
+      <c r="E3" s="17" t="n"/>
       <c r="F3" s="7" t="n"/>
-      <c r="G3" s="7" t="n"/>
-      <c r="H3" s="9" t="n">
+      <c r="G3" s="18" t="n"/>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="9" t="n">
         <v>66</v>
       </c>
-      <c r="I3" s="10" t="n">
+      <c r="J3" s="19" t="n">
         <v>2525000</v>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>Minhas Ladiwalla</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>3550 Labounty Drive</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>Oceanside</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>Zeenat Ladiwalla</t>
         </is>
       </c>
-      <c r="P3" s="6" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
         <is>
           <t>Allen CA</t>
         </is>
       </c>
-      <c r="Q3" s="6" t="inlineStr">
+      <c r="R3" s="6" t="inlineStr">
         <is>
           <t>M. Neil Solarz</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr">
+      <c r="S3" s="6" t="inlineStr">
         <is>
           <t>(310) 553-8844 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S3" s="11" t="inlineStr">
+      <c r="T3" s="11" t="inlineStr">
         <is>
           <t>29mo old; $1M+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -972,63 +1027,64 @@
         </is>
       </c>
       <c r="B4" s="7" t="n"/>
-      <c r="C4" s="8" t="n"/>
+      <c r="C4" s="17" t="n"/>
       <c r="D4" s="7" t="n"/>
-      <c r="E4" s="8" t="n"/>
+      <c r="E4" s="17" t="n"/>
       <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="9" t="n">
+      <c r="G4" s="18" t="n"/>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="9" t="n">
         <v>61</v>
       </c>
-      <c r="I4" s="10" t="n">
+      <c r="J4" s="19" t="n">
         <v>2090678</v>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Anna Luise Manicke-Schulmann aka Anna L. Manicke aka Anna L. Schulmann</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>2019 Cordero Road</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>Del Mar</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O4" s="6" t="inlineStr">
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>Tatiana Tonekaboni</t>
         </is>
       </c>
-      <c r="P4" s="6" t="inlineStr">
+      <c r="Q4" s="6" t="inlineStr">
         <is>
           <t>Hendersonville TN</t>
         </is>
       </c>
-      <c r="Q4" s="6" t="inlineStr">
+      <c r="R4" s="6" t="inlineStr">
         <is>
           <t>Steven F. Bliss</t>
         </is>
       </c>
-      <c r="R4" s="6" t="inlineStr">
+      <c r="S4" s="6" t="inlineStr">
         <is>
           <t>(951) 223-7000</t>
         </is>
       </c>
-      <c r="S4" s="11" t="inlineStr">
+      <c r="T4" s="11" t="inlineStr">
         <is>
           <t>26mo old; $1M+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -1040,64 +1096,89 @@
           <t>24PE001330C</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="9" t="n">
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Accounting hearing - Amended Report and First and Final Account (ROA 28)</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
+        <is>
+          <t>Moving toward final distribution, hearing 8/25/2026. Co-administrators Jane Hudson and Marion Richards with shared counsel; four additional interested parties, so consent may be slow.</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="I5" s="10" t="n">
+      <c r="J5" s="19" t="n">
         <v>2173003</v>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>Samuel Robert Thomas Richards</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>1127 Reed Ave. Apt. 6</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>Jane R. Hudson and Marion K. Richards</t>
         </is>
       </c>
-      <c r="P5" s="6" t="inlineStr">
+      <c r="Q5" s="6" t="inlineStr">
         <is>
           <t>Warrenton NC</t>
         </is>
       </c>
-      <c r="Q5" s="6" t="inlineStr">
+      <c r="R5" s="6" t="inlineStr">
         <is>
           <t>Maya M. Pinchman</t>
         </is>
       </c>
-      <c r="R5" s="6" t="inlineStr">
+      <c r="S5" s="6" t="inlineStr">
         <is>
           <t>800-836-1124 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S5" s="11" t="inlineStr">
+      <c r="T5" s="11" t="inlineStr">
         <is>
           <t>26mo old; $1M+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -1110,63 +1191,64 @@
         </is>
       </c>
       <c r="B6" s="7" t="n"/>
-      <c r="C6" s="8" t="n"/>
+      <c r="C6" s="17" t="n"/>
       <c r="D6" s="7" t="n"/>
-      <c r="E6" s="8" t="n"/>
+      <c r="E6" s="17" t="n"/>
       <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="9" t="n">
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="I6" s="10" t="n">
+      <c r="J6" s="19" t="n">
         <v>2084303</v>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Ila K. Margagliano (aka Ila Kathleen Margagliano)</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>5219 Clairemont Mesa Blvd.</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O6" s="6" t="inlineStr">
+      <c r="P6" s="6" t="inlineStr">
         <is>
           <t>Joni Jugler</t>
         </is>
       </c>
-      <c r="P6" s="6" t="inlineStr">
+      <c r="Q6" s="6" t="inlineStr">
         <is>
           <t>Colorado Springs CO</t>
         </is>
       </c>
-      <c r="Q6" s="6" t="inlineStr">
+      <c r="R6" s="6" t="inlineStr">
         <is>
           <t>Erin C. Foley</t>
         </is>
       </c>
-      <c r="R6" s="6" t="inlineStr">
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>619-284-2444</t>
         </is>
       </c>
-      <c r="S6" s="11" t="inlineStr">
+      <c r="T6" s="11" t="inlineStr">
         <is>
           <t>26mo old; $1M+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -1179,63 +1261,64 @@
         </is>
       </c>
       <c r="B7" s="7" t="n"/>
-      <c r="C7" s="8" t="n"/>
+      <c r="C7" s="17" t="n"/>
       <c r="D7" s="7" t="n"/>
-      <c r="E7" s="8" t="n"/>
+      <c r="E7" s="17" t="n"/>
       <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="9" t="n">
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="I7" s="10" t="n">
+      <c r="J7" s="19" t="n">
         <v>468800</v>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>JESSE JAE SOO PARK</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>2540 Clairemont Drive Unit 108</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O7" s="6" t="inlineStr">
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>Jennifer P. Fasano</t>
         </is>
       </c>
-      <c r="P7" s="6" t="inlineStr">
+      <c r="Q7" s="6" t="inlineStr">
         <is>
           <t>Las Vegas NV</t>
         </is>
       </c>
-      <c r="Q7" s="6" t="inlineStr">
+      <c r="R7" s="6" t="inlineStr">
         <is>
           <t>Pro Per</t>
         </is>
       </c>
-      <c r="R7" s="6" t="inlineStr">
+      <c r="S7" s="6" t="inlineStr">
         <is>
           <t>702-499-9378 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S7" s="11" t="inlineStr">
+      <c r="T7" s="11" t="inlineStr">
         <is>
           <t>26mo old; $350k+ equity; vacant/absentee; self-represented; out-of-county heir</t>
         </is>
@@ -1247,64 +1330,89 @@
           <t>24PE001624C</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="9" t="n">
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>46219</v>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Notice of Hearing (ROA 27)</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>46461</v>
+      </c>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>YES - 2 notices (3/14/25, 5/29/26)</t>
+        </is>
+      </c>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>Court issued two Notices of Failure to Perform Duties. Letters expired 4/30/2026 and were not renewed. Next review not until Mar 2027. Executor represented by an Arizona attorney.</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="n">
         <v>59</v>
       </c>
-      <c r="I8" s="10" t="n">
+      <c r="J8" s="19" t="n">
         <v>1552181</v>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>DORA V. ROSCHEFSKI</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>3850 Valley Vista Rd.</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
         <is>
           <t>Bonita</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O8" s="6" t="inlineStr">
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>James Paul Roschefski</t>
         </is>
       </c>
-      <c r="P8" s="6" t="inlineStr">
+      <c r="Q8" s="6" t="inlineStr">
         <is>
           <t>Waterford MI</t>
         </is>
       </c>
-      <c r="Q8" s="6" t="inlineStr">
+      <c r="R8" s="6" t="inlineStr">
         <is>
           <t>Donald F. Coats, Jr.</t>
         </is>
       </c>
-      <c r="R8" s="6" t="inlineStr">
+      <c r="S8" s="6" t="inlineStr">
         <is>
           <t>(619) 838-3259 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S8" s="11" t="inlineStr">
+      <c r="T8" s="11" t="inlineStr">
         <is>
           <t>25mo old; $1M+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -1316,64 +1424,89 @@
           <t>24PE000377C</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="9" t="n">
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>46101</v>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>Letters Extended/Reissued to 8/11/2026 (ROA 120)</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>46245</v>
+      </c>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="25" t="inlineStr">
+        <is>
+          <t>YES - OSC re sanctions</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>STRONGEST DISTRESS SIGNAL. OSC issued 3/19/2026 over the administrator distributing estate assets without court authorization, proposing $1,500 sanctions and revocation of Letters. Administrator is self-represented. Public Administrator is an interested party. 120 docket entries.</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="n">
         <v>58</v>
       </c>
-      <c r="I9" s="10" t="n">
+      <c r="J9" s="19" t="n">
         <v>203776</v>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Jeanne D. Willis</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>2825 3rd Ave. #208</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M9" s="6" t="inlineStr">
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="O9" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr">
+      <c r="P9" s="6" t="inlineStr">
         <is>
           <t>Paul Ellington Willis</t>
         </is>
       </c>
-      <c r="P9" s="6" t="inlineStr">
+      <c r="Q9" s="6" t="inlineStr">
         <is>
           <t>Lodi CA</t>
         </is>
       </c>
-      <c r="Q9" s="6" t="inlineStr">
+      <c r="R9" s="6" t="inlineStr">
         <is>
           <t>Pro Per</t>
         </is>
       </c>
-      <c r="R9" s="6" t="inlineStr">
+      <c r="S9" s="6" t="inlineStr">
         <is>
           <t>(760) 201-5641 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S9" s="11" t="inlineStr">
+      <c r="T9" s="11" t="inlineStr">
         <is>
           <t>28mo old; $150k+ equity; vacant/absentee; self-represented; out-of-county heir</t>
         </is>
@@ -1385,64 +1518,89 @@
           <t>24PE001705C</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="9" t="n">
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>Notice of Hearing (ROA 54)</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>46231</v>
+      </c>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>YES - 2 notices (1/27/25, 4/14/26)</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>CONTESTED. Competing petitions between Charlene Brown and Terri Gascon, plus a civil complaint alleging breach of contract, promissory estoppel, fraud and unjust enrichment. Inventory and Appraisal filed as Final $0.00. Letters expired 3/25/2026. Two law firms involved - a difficult approach.</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="n">
         <v>55</v>
       </c>
-      <c r="I10" s="10" t="n">
+      <c r="J10" s="19" t="n">
         <v>3162994</v>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>Charles Terry Brown</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>5724 Dolphin PI.</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="M10" s="6" t="inlineStr">
         <is>
           <t>La Jolla</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr">
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>OWNER OCCUPIED</t>
         </is>
       </c>
-      <c r="N10" s="6" t="inlineStr">
+      <c r="O10" s="6" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="O10" s="6" t="inlineStr">
+      <c r="P10" s="6" t="inlineStr">
         <is>
           <t>Terri Lynn Gascon</t>
         </is>
       </c>
-      <c r="P10" s="6" t="inlineStr">
+      <c r="Q10" s="6" t="inlineStr">
         <is>
           <t>Bend OR</t>
         </is>
       </c>
-      <c r="Q10" s="6" t="inlineStr">
+      <c r="R10" s="6" t="inlineStr">
         <is>
           <t>Casey A. Reagan</t>
         </is>
       </c>
-      <c r="R10" s="6" t="inlineStr">
+      <c r="S10" s="6" t="inlineStr">
         <is>
           <t>310-444-9060 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S10" s="11" t="inlineStr">
+      <c r="T10" s="11" t="inlineStr">
         <is>
           <t>25mo old; $1M+ equity; limited authority (court confirmation); out-of-county heir</t>
         </is>
@@ -1455,59 +1613,60 @@
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
-      <c r="C11" s="8" t="n"/>
+      <c r="C11" s="17" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="E11" s="17" t="n"/>
       <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="9" t="n">
+      <c r="G11" s="18" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="9" t="n">
         <v>54</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="J11" s="19" t="n">
         <v>1178273</v>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>Jimmie Ray Haymon</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>8530 Nelson Way</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>Escondido</t>
         </is>
       </c>
-      <c r="M11" s="6" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N11" s="6" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O11" s="6" t="inlineStr">
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>Dorothy Cavallo</t>
         </is>
       </c>
-      <c r="P11" s="6" t="inlineStr">
+      <c r="Q11" s="6" t="inlineStr">
         <is>
           <t>San Marcos CA</t>
         </is>
       </c>
-      <c r="Q11" s="6" t="inlineStr">
+      <c r="R11" s="6" t="inlineStr">
         <is>
           <t>Alan Mansfield</t>
         </is>
       </c>
-      <c r="R11" s="6" t="n"/>
-      <c r="S11" s="11" t="inlineStr">
+      <c r="S11" s="6" t="n"/>
+      <c r="T11" s="11" t="inlineStr">
         <is>
           <t>25mo old; $1M+ equity; vacant/absentee; heir not at property</t>
         </is>
@@ -1520,63 +1679,64 @@
         </is>
       </c>
       <c r="B12" s="7" t="n"/>
-      <c r="C12" s="8" t="n"/>
+      <c r="C12" s="17" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="8" t="n"/>
+      <c r="E12" s="17" t="n"/>
       <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="9" t="n">
+      <c r="G12" s="18" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="9" t="n">
         <v>54</v>
       </c>
-      <c r="I12" s="10" t="n">
+      <c r="J12" s="19" t="n">
         <v>475000</v>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>GLADYS MCMULLEN</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>689 Crested Butte Street</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="M12" s="6" t="inlineStr">
         <is>
           <t>Chula Vista</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr">
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N12" s="6" t="inlineStr">
+      <c r="O12" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O12" s="6" t="inlineStr">
+      <c r="P12" s="6" t="inlineStr">
         <is>
           <t>Laura Lewis</t>
         </is>
       </c>
-      <c r="P12" s="6" t="inlineStr">
+      <c r="Q12" s="6" t="inlineStr">
         <is>
           <t>Woodbridge VA</t>
         </is>
       </c>
-      <c r="Q12" s="6" t="inlineStr">
+      <c r="R12" s="6" t="inlineStr">
         <is>
           <t>Benjamin S. Green</t>
         </is>
       </c>
-      <c r="R12" s="6" t="inlineStr">
+      <c r="S12" s="6" t="inlineStr">
         <is>
           <t>619-425-4020</t>
         </is>
       </c>
-      <c r="S12" s="11" t="inlineStr">
+      <c r="T12" s="11" t="inlineStr">
         <is>
           <t>29mo old; $350k+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -1588,56 +1748,81 @@
           <t>24PE000842C</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="9" t="n">
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>Review Hearing - failure to perform duties re: final accounting (ROA 26)</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>46282</v>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" s="25" t="inlineStr">
+        <is>
+          <t>YES - hearing set on it</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr">
+        <is>
+          <t>Self-represented executor who is visibly struggling - two filings rejected by the clerk (1/7/2026 and 1/28/2026) and a standing Failure to Perform Duties review. No attorney of record. Best fit for a help-oriented approach.</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="n">
         <v>53</v>
       </c>
-      <c r="I13" s="10" t="n">
+      <c r="J13" s="19" t="n">
         <v>679000</v>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Kenneth Leland Walters AKA Kenneth Leland Waiters Jr.</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>9330 Gregory St.</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>La Mesa</t>
         </is>
       </c>
-      <c r="M13" s="6" t="n"/>
-      <c r="N13" s="6" t="inlineStr">
+      <c r="N13" s="6" t="n"/>
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O13" s="6" t="inlineStr">
+      <c r="P13" s="6" t="inlineStr">
         <is>
           <t>Cary C. Crane</t>
         </is>
       </c>
-      <c r="P13" s="6" t="inlineStr">
+      <c r="Q13" s="6" t="inlineStr">
         <is>
           <t>Idaho Springs CO</t>
         </is>
       </c>
-      <c r="Q13" s="6" t="inlineStr">
+      <c r="R13" s="6" t="inlineStr">
         <is>
           <t>Pro Per</t>
         </is>
       </c>
-      <c r="R13" s="6" t="n"/>
-      <c r="S13" s="11" t="inlineStr">
+      <c r="S13" s="6" t="n"/>
+      <c r="T13" s="11" t="inlineStr">
         <is>
           <t>27mo old; $600k+ equity; self-represented; out-of-county heir</t>
         </is>
@@ -1649,64 +1834,87 @@
           <t>24PE000357C</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="9" t="n">
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="n">
+        <v>46086</v>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>Ex Parte Petition for Final Discharge and Order (ROA 40)</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G14" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="30" t="inlineStr">
+        <is>
+          <t>CLOSED. Final distribution approved 1/7/2026, final discharge filed 3/5/2026. Remove from pipeline.</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="n">
         <v>51</v>
       </c>
-      <c r="I14" s="10" t="n">
+      <c r="J14" s="19" t="n">
         <v>2500000</v>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>ESTHER COOPER aka ESTEE COOPER</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>7143 Almaden Lane</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="M14" s="6" t="inlineStr">
         <is>
           <t>Carlsbad</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>OWNER OCCUPIED</t>
         </is>
       </c>
-      <c r="N14" s="6" t="inlineStr">
+      <c r="O14" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O14" s="6" t="inlineStr">
+      <c r="P14" s="6" t="inlineStr">
         <is>
           <t>SANDY L. SOLOMON</t>
         </is>
       </c>
-      <c r="P14" s="6" t="inlineStr">
+      <c r="Q14" s="6" t="inlineStr">
         <is>
           <t>Reading PA</t>
         </is>
       </c>
-      <c r="Q14" s="6" t="inlineStr">
+      <c r="R14" s="6" t="inlineStr">
         <is>
           <t>Stuart N. Chelin</t>
         </is>
       </c>
-      <c r="R14" s="6" t="inlineStr">
+      <c r="S14" s="6" t="inlineStr">
         <is>
           <t>(310) 556-9664</t>
         </is>
       </c>
-      <c r="S14" s="11" t="inlineStr">
+      <c r="T14" s="11" t="inlineStr">
         <is>
           <t>28mo old; $1M+ equity; out-of-county heir</t>
         </is>
@@ -1718,64 +1926,87 @@
           <t>24PE000332C</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="9" t="n">
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>45996</v>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Proof of Service (ROA 47)</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>MOST DORMANT of the group - nothing filed since Dec 2025, nearly eight months, and no hearing on calendar. Letters were extended to 10/17/2027, so the administrator is planning a long runway.</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="n">
         <v>51</v>
       </c>
-      <c r="I15" s="10" t="n">
+      <c r="J15" s="19" t="n">
         <v>1827500</v>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>KATHLEEN ANN TURNER aka KATHY A. TURNER</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>9462 Doheny Road</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>Santee</t>
         </is>
       </c>
-      <c r="M15" s="6" t="inlineStr">
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>OWNER OCCUPIED</t>
         </is>
       </c>
-      <c r="N15" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O15" s="6" t="inlineStr">
+      <c r="P15" s="6" t="inlineStr">
         <is>
           <t>EILEEN NUNLEY</t>
         </is>
       </c>
-      <c r="P15" s="6" t="inlineStr">
+      <c r="Q15" s="6" t="inlineStr">
         <is>
           <t>FALMOUTH ME</t>
         </is>
       </c>
-      <c r="Q15" s="6" t="inlineStr">
+      <c r="R15" s="6" t="inlineStr">
         <is>
           <t>MIRANDA C. FRANKS</t>
         </is>
       </c>
-      <c r="R15" s="6" t="inlineStr">
+      <c r="S15" s="6" t="inlineStr">
         <is>
           <t>619-660-0520 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S15" s="11" t="inlineStr">
+      <c r="T15" s="11" t="inlineStr">
         <is>
           <t>28mo old; $1M+ equity; out-of-county heir</t>
         </is>
@@ -1788,63 +2019,64 @@
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
-      <c r="C16" s="8" t="n"/>
+      <c r="C16" s="17" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="8" t="n"/>
+      <c r="E16" s="17" t="n"/>
       <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="9" t="n">
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="9" t="n">
         <v>51</v>
       </c>
-      <c r="I16" s="10" t="n">
+      <c r="J16" s="19" t="n">
         <v>1000182</v>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Keith L. Wasser</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>4649 El Penon Way</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M16" s="6" t="inlineStr">
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>OWNER OCCUPIED</t>
         </is>
       </c>
-      <c r="N16" s="6" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O16" s="6" t="inlineStr">
+      <c r="P16" s="6" t="inlineStr">
         <is>
           <t>Monica Famularo</t>
         </is>
       </c>
-      <c r="P16" s="6" t="inlineStr">
+      <c r="Q16" s="6" t="inlineStr">
         <is>
           <t>Virginia Beach VA</t>
         </is>
       </c>
-      <c r="Q16" s="6" t="inlineStr">
+      <c r="R16" s="6" t="inlineStr">
         <is>
           <t>Julia A. Solaegui</t>
         </is>
       </c>
-      <c r="R16" s="6" t="inlineStr">
+      <c r="S16" s="6" t="inlineStr">
         <is>
           <t>(619) 588-2828 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S16" s="11" t="inlineStr">
+      <c r="T16" s="11" t="inlineStr">
         <is>
           <t>28mo old; $1M+ equity; out-of-county heir</t>
         </is>
@@ -1856,64 +2088,87 @@
           <t>24PE001060C</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="9" t="n">
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>46061</v>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>System Generated Notice E-mailed (ROA 28)</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="24" t="inlineStr">
+        <is>
+          <t>Quiet since Feb 2026 - roughly five months with no filings and no hearing set. Administrator and counsel are both in St. George, Utah. Letters run to 12/11/2026.</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="I17" s="10" t="n">
+      <c r="J17" s="19" t="n">
         <v>485167</v>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>Jerry Michael Soderlling</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>2655 Joann Drive</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
         <is>
           <t>Oceanside</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="N17" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N17" s="6" t="inlineStr">
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O17" s="6" t="inlineStr">
+      <c r="P17" s="6" t="inlineStr">
         <is>
           <t>Joanna Sidney Gomlicker</t>
         </is>
       </c>
-      <c r="P17" s="6" t="inlineStr">
+      <c r="Q17" s="6" t="inlineStr">
         <is>
           <t>Stuart FL</t>
         </is>
       </c>
-      <c r="Q17" s="6" t="inlineStr">
+      <c r="R17" s="6" t="inlineStr">
         <is>
           <t>E. LAWRENCE BROCK</t>
         </is>
       </c>
-      <c r="R17" s="6" t="inlineStr">
+      <c r="S17" s="6" t="inlineStr">
         <is>
           <t>435-688-9231 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S17" s="11" t="inlineStr">
+      <c r="T17" s="11" t="inlineStr">
         <is>
           <t>26mo old; $350k+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -1926,63 +2181,64 @@
         </is>
       </c>
       <c r="B18" s="7" t="n"/>
-      <c r="C18" s="8" t="n"/>
+      <c r="C18" s="17" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="8" t="n"/>
+      <c r="E18" s="17" t="n"/>
       <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="9" t="n">
+      <c r="G18" s="18" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="I18" s="10" t="n">
+      <c r="J18" s="19" t="n">
         <v>432000</v>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>ESTA LYN TEMPLE BURKE</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>7760 MARGERUM AVE., UNIT 126</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="M18" s="6" t="inlineStr">
         <is>
           <t>SAN DIEGO</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr">
+      <c r="N18" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N18" s="6" t="inlineStr">
+      <c r="O18" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O18" s="6" t="inlineStr">
+      <c r="P18" s="6" t="inlineStr">
         <is>
           <t>ZACHARY STEPHEN LITTEN</t>
         </is>
       </c>
-      <c r="P18" s="6" t="inlineStr">
+      <c r="Q18" s="6" t="inlineStr">
         <is>
           <t>NORTH CHESTERFIELD VA</t>
         </is>
       </c>
-      <c r="Q18" s="6" t="inlineStr">
+      <c r="R18" s="6" t="inlineStr">
         <is>
           <t>RICH GAINES</t>
         </is>
       </c>
-      <c r="R18" s="6" t="inlineStr">
+      <c r="S18" s="6" t="inlineStr">
         <is>
           <t>760-931-9923</t>
         </is>
       </c>
-      <c r="S18" s="11" t="inlineStr">
+      <c r="T18" s="11" t="inlineStr">
         <is>
           <t>27mo old; $350k+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -1994,64 +2250,89 @@
           <t>24PE001744C</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="9" t="n">
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>Notice of Hearing (ROA 43)</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>46413</v>
+      </c>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
+        <is>
+          <t>WINDING DOWN. Report and Accounting plus Petition for Final Distribution filed 6/29/2026. This estate is on its way out - lowest priority of the open cases.</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="I19" s="10" t="n">
+      <c r="J19" s="19" t="n">
         <v>155848</v>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Jason Hideo Burke, aka Jason Burke, aka Jason H. Burke</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>2108 3rd Ave, Unit 1</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="P19" s="6" t="inlineStr">
         <is>
           <t>Connor Burke</t>
         </is>
       </c>
-      <c r="P19" s="6" t="inlineStr">
+      <c r="Q19" s="6" t="inlineStr">
         <is>
           <t>Brick NJ</t>
         </is>
       </c>
-      <c r="Q19" s="6" t="inlineStr">
+      <c r="R19" s="6" t="inlineStr">
         <is>
           <t>Weily Yang</t>
         </is>
       </c>
-      <c r="R19" s="6" t="inlineStr">
+      <c r="S19" s="6" t="inlineStr">
         <is>
           <t>714-573-7149</t>
         </is>
       </c>
-      <c r="S19" s="11" t="inlineStr">
+      <c r="T19" s="11" t="inlineStr">
         <is>
           <t>24mo old; $150k+ equity; vacant/absentee; limited authority (court confirmation); out-of-county heir</t>
         </is>
@@ -2064,63 +2345,64 @@
         </is>
       </c>
       <c r="B20" s="7" t="n"/>
-      <c r="C20" s="8" t="n"/>
+      <c r="C20" s="17" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="8" t="n"/>
+      <c r="E20" s="17" t="n"/>
       <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="9" t="n">
+      <c r="G20" s="18" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="9" t="n">
         <v>48</v>
       </c>
-      <c r="I20" s="10" t="n">
+      <c r="J20" s="19" t="n">
         <v>390000</v>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Betty Simmons</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>1968 Canyas Drive,Unit 6</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
         <is>
           <t>Chula Vista</t>
         </is>
       </c>
-      <c r="M20" s="6" t="inlineStr">
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N20" s="6" t="inlineStr">
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O20" s="6" t="inlineStr">
+      <c r="P20" s="6" t="inlineStr">
         <is>
           <t>ALEC B. SIMMONS, Jr.</t>
         </is>
       </c>
-      <c r="P20" s="6" t="inlineStr">
+      <c r="Q20" s="6" t="inlineStr">
         <is>
           <t>Tempe AZ</t>
         </is>
       </c>
-      <c r="Q20" s="6" t="inlineStr">
+      <c r="R20" s="6" t="inlineStr">
         <is>
           <t>ELAINE M. BALOK</t>
         </is>
       </c>
-      <c r="R20" s="6" t="inlineStr">
+      <c r="S20" s="6" t="inlineStr">
         <is>
           <t>619-337-6700</t>
         </is>
       </c>
-      <c r="S20" s="11" t="inlineStr">
+      <c r="T20" s="11" t="inlineStr">
         <is>
           <t>25mo old; $350k+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -2133,63 +2415,64 @@
         </is>
       </c>
       <c r="B21" s="7" t="n"/>
-      <c r="C21" s="8" t="n"/>
+      <c r="C21" s="17" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="8" t="n"/>
+      <c r="E21" s="17" t="n"/>
       <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="9" t="n">
+      <c r="G21" s="18" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I21" s="10" t="n">
+      <c r="J21" s="19" t="n">
         <v>15459147</v>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>ROSS STANFORD GILBERT</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>101 Border Avenue</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="M21" s="6" t="inlineStr">
         <is>
           <t>Del Mar</t>
         </is>
       </c>
-      <c r="M21" s="6" t="inlineStr">
+      <c r="N21" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N21" s="6" t="inlineStr">
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O21" s="6" t="inlineStr">
+      <c r="P21" s="6" t="inlineStr">
         <is>
           <t>Mary-K. Gilbert, also known as Mary Katherine Gilb</t>
         </is>
       </c>
-      <c r="P21" s="6" t="inlineStr">
+      <c r="Q21" s="6" t="inlineStr">
         <is>
           <t>Del Mar CA</t>
         </is>
       </c>
-      <c r="Q21" s="6" t="inlineStr">
+      <c r="R21" s="6" t="inlineStr">
         <is>
           <t>Philip M. Savage, IV and David D. Werner</t>
         </is>
       </c>
-      <c r="R21" s="6" t="inlineStr">
+      <c r="S21" s="6" t="inlineStr">
         <is>
           <t>909-890-4499</t>
         </is>
       </c>
-      <c r="S21" s="11" t="inlineStr">
+      <c r="T21" s="11" t="inlineStr">
         <is>
           <t>25mo old; $1M+ equity; vacant/absentee</t>
         </is>
@@ -2201,60 +2484,85 @@
           <t>24PE001572C</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="9" t="n">
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="n">
+        <v>46181</v>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Declaration - Withdrawal of Wells Fargo creditor claim (ROA 37)</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>46440</v>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="25" t="inlineStr">
+        <is>
+          <t>YES - hearing set on it</t>
+        </is>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
+        <is>
+          <t>Court has set a Failure to Perform Duties review. Corrected Final Inventory and Appraisal filed 4/30/2026, so valuation work is done but distribution is not. Wells Fargo withdrew its creditor claim.</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I22" s="10" t="n">
+      <c r="J22" s="19" t="n">
         <v>1641172</v>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>GEORGE WALTHER-MEADE</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>419 Milagrosa Circle</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="M22" s="6" t="inlineStr">
         <is>
           <t>Chula Vista</t>
         </is>
       </c>
-      <c r="M22" s="6" t="inlineStr">
+      <c r="N22" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N22" s="6" t="inlineStr">
+      <c r="O22" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O22" s="6" t="inlineStr">
+      <c r="P22" s="6" t="inlineStr">
         <is>
           <t>George M. Walther-Meade</t>
         </is>
       </c>
-      <c r="P22" s="6" t="inlineStr">
+      <c r="Q22" s="6" t="inlineStr">
         <is>
           <t>Chula Vista CA</t>
         </is>
       </c>
-      <c r="Q22" s="6" t="inlineStr">
+      <c r="R22" s="6" t="inlineStr">
         <is>
           <t>John W. Melvin</t>
         </is>
       </c>
-      <c r="R22" s="6" t="n"/>
-      <c r="S22" s="11" t="inlineStr">
+      <c r="S22" s="6" t="n"/>
+      <c r="T22" s="11" t="inlineStr">
         <is>
           <t>25mo old; $1M+ equity; vacant/absentee</t>
         </is>
@@ -2267,63 +2575,64 @@
         </is>
       </c>
       <c r="B23" s="7" t="n"/>
-      <c r="C23" s="8" t="n"/>
+      <c r="C23" s="17" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="8" t="n"/>
+      <c r="E23" s="17" t="n"/>
       <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="9" t="n">
+      <c r="G23" s="18" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I23" s="10" t="n">
+      <c r="J23" s="19" t="n">
         <v>1294988</v>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>Thomas B. Galligan</t>
         </is>
       </c>
-      <c r="K23" s="6" t="inlineStr">
+      <c r="L23" s="6" t="inlineStr">
         <is>
           <t>2163 Calle Frescot</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr">
+      <c r="M23" s="6" t="inlineStr">
         <is>
           <t>La Jolla</t>
         </is>
       </c>
-      <c r="M23" s="6" t="inlineStr">
+      <c r="N23" s="6" t="inlineStr">
         <is>
           <t>OWNER OCCUPIED</t>
         </is>
       </c>
-      <c r="N23" s="6" t="inlineStr">
+      <c r="O23" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O23" s="6" t="inlineStr">
+      <c r="P23" s="6" t="inlineStr">
         <is>
           <t>Patricia M. Galligan</t>
         </is>
       </c>
-      <c r="P23" s="6" t="inlineStr">
+      <c r="Q23" s="6" t="inlineStr">
         <is>
           <t>La Jolla CA</t>
         </is>
       </c>
-      <c r="Q23" s="6" t="inlineStr">
+      <c r="R23" s="6" t="inlineStr">
         <is>
           <t>Pro Per</t>
         </is>
       </c>
-      <c r="R23" s="6" t="inlineStr">
+      <c r="S23" s="6" t="inlineStr">
         <is>
           <t>858-643-5700 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S23" s="11" t="inlineStr">
+      <c r="T23" s="11" t="inlineStr">
         <is>
           <t>26mo old; $1M+ equity; self-represented</t>
         </is>
@@ -2335,64 +2644,87 @@
           <t>24PE000954C</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="9" t="n">
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>Letters Extended/Reissued to 4/30/2027 (ROA 101)</t>
+        </is>
+      </c>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G24" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" s="24" t="inlineStr">
+        <is>
+          <t>CONTESTED among family - three competing petitioners (Laurvick, Frederic Nevins, Patricia Nevins) with separate counsel. American Express is a claimant. Letters extended all the way to Apr 2027, which signals the court expects this to run long.</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I24" s="10" t="n">
+      <c r="J24" s="19" t="n">
         <v>1262000</v>
       </c>
-      <c r="J24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Jeffrey Benjamin Nevins</t>
         </is>
       </c>
-      <c r="K24" s="6" t="inlineStr">
+      <c r="L24" s="6" t="inlineStr">
         <is>
           <t>4316 Haines Street</t>
         </is>
       </c>
-      <c r="L24" s="6" t="inlineStr">
+      <c r="M24" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M24" s="6" t="inlineStr">
+      <c r="N24" s="6" t="inlineStr">
         <is>
           <t>OWNER OCCUPIED</t>
         </is>
       </c>
-      <c r="N24" s="6" t="inlineStr">
+      <c r="O24" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O24" s="6" t="inlineStr">
+      <c r="P24" s="6" t="inlineStr">
         <is>
           <t>Frederic Nevins</t>
         </is>
       </c>
-      <c r="P24" s="6" t="inlineStr">
+      <c r="Q24" s="6" t="inlineStr">
         <is>
           <t>Port Washington NY</t>
         </is>
       </c>
-      <c r="Q24" s="6" t="inlineStr">
+      <c r="R24" s="6" t="inlineStr">
         <is>
           <t>James F. Watts</t>
         </is>
       </c>
-      <c r="R24" s="6" t="inlineStr">
+      <c r="S24" s="6" t="inlineStr">
         <is>
           <t>858-481-2880 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S24" s="11" t="inlineStr">
+      <c r="T24" s="11" t="inlineStr">
         <is>
           <t>27mo old; $1M+ equity; out-of-county heir</t>
         </is>
@@ -2405,59 +2737,60 @@
         </is>
       </c>
       <c r="B25" s="7" t="n"/>
-      <c r="C25" s="8" t="n"/>
+      <c r="C25" s="17" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="8" t="n"/>
+      <c r="E25" s="17" t="n"/>
       <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="9" t="n">
+      <c r="G25" s="18" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I25" s="10" t="n">
+      <c r="J25" s="19" t="n">
         <v>1150000</v>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>Henry Hingwhee Lin aka Henry Hing-Whee Lin aka Henry Hing Whee Lin</t>
         </is>
       </c>
-      <c r="K25" s="6" t="inlineStr">
+      <c r="L25" s="6" t="inlineStr">
         <is>
           <t>12719 Robison Boulevard #9</t>
         </is>
       </c>
-      <c r="L25" s="6" t="inlineStr">
+      <c r="M25" s="6" t="inlineStr">
         <is>
           <t>Poway</t>
         </is>
       </c>
-      <c r="M25" s="6" t="n"/>
-      <c r="N25" s="6" t="inlineStr">
+      <c r="N25" s="6" t="n"/>
+      <c r="O25" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O25" s="6" t="inlineStr">
+      <c r="P25" s="6" t="inlineStr">
         <is>
           <t>Yihwen Lin</t>
         </is>
       </c>
-      <c r="P25" s="6" t="inlineStr">
+      <c r="Q25" s="6" t="inlineStr">
         <is>
           <t>Covina CA</t>
         </is>
       </c>
-      <c r="Q25" s="6" t="inlineStr">
+      <c r="R25" s="6" t="inlineStr">
         <is>
           <t>Daniel K. Printz and Deborah Chew</t>
         </is>
       </c>
-      <c r="R25" s="6" t="inlineStr">
+      <c r="S25" s="6" t="inlineStr">
         <is>
           <t>858-519-8020</t>
         </is>
       </c>
-      <c r="S25" s="11" t="inlineStr">
+      <c r="T25" s="11" t="inlineStr">
         <is>
           <t>26mo old; $1M+ equity; out-of-county heir</t>
         </is>
@@ -2470,59 +2803,60 @@
         </is>
       </c>
       <c r="B26" s="7" t="n"/>
-      <c r="C26" s="8" t="n"/>
+      <c r="C26" s="17" t="n"/>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="8" t="n"/>
+      <c r="E26" s="17" t="n"/>
       <c r="F26" s="7" t="n"/>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="9" t="n">
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I26" s="10" t="n">
+      <c r="J26" s="19" t="n">
         <v>1000000</v>
       </c>
-      <c r="J26" s="6" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>Melchor Balaguer</t>
         </is>
       </c>
-      <c r="K26" s="6" t="inlineStr">
+      <c r="L26" s="6" t="inlineStr">
         <is>
           <t>230 W. Laurel Street  #503</t>
         </is>
       </c>
-      <c r="L26" s="6" t="inlineStr">
+      <c r="M26" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M26" s="6" t="inlineStr">
+      <c r="N26" s="6" t="inlineStr">
         <is>
           <t>OWNER OCCUPIED</t>
         </is>
       </c>
-      <c r="N26" s="6" t="inlineStr">
+      <c r="O26" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O26" s="6" t="inlineStr">
+      <c r="P26" s="6" t="inlineStr">
         <is>
           <t>Ellen Marie Balaguer</t>
         </is>
       </c>
-      <c r="P26" s="6" t="inlineStr">
+      <c r="Q26" s="6" t="inlineStr">
         <is>
           <t>Greenwood Village CO</t>
         </is>
       </c>
-      <c r="Q26" s="6" t="inlineStr">
+      <c r="R26" s="6" t="inlineStr">
         <is>
           <t>Kristan Shepard and Tamie Humphreys</t>
         </is>
       </c>
-      <c r="R26" s="6" t="n"/>
-      <c r="S26" s="11" t="inlineStr">
+      <c r="S26" s="6" t="n"/>
+      <c r="T26" s="11" t="inlineStr">
         <is>
           <t>26mo old; $1M+ equity; out-of-county heir</t>
         </is>
@@ -2535,63 +2869,64 @@
         </is>
       </c>
       <c r="B27" s="7" t="n"/>
-      <c r="C27" s="8" t="n"/>
+      <c r="C27" s="17" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="8" t="n"/>
+      <c r="E27" s="17" t="n"/>
       <c r="F27" s="7" t="n"/>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="9" t="n">
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I27" s="10" t="n">
+      <c r="J27" s="19" t="n">
         <v>454430</v>
       </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>JOHN VINCENT KAISER JR AKA JOHN V. KAISER JR.</t>
         </is>
       </c>
-      <c r="K27" s="6" t="inlineStr">
+      <c r="L27" s="6" t="inlineStr">
         <is>
           <t>1077 Glenhill Road</t>
         </is>
       </c>
-      <c r="L27" s="6" t="inlineStr">
+      <c r="M27" s="6" t="inlineStr">
         <is>
           <t>El Cajon</t>
         </is>
       </c>
-      <c r="M27" s="6" t="inlineStr">
+      <c r="N27" s="6" t="inlineStr">
         <is>
           <t>ABSENTEE</t>
         </is>
       </c>
-      <c r="N27" s="6" t="inlineStr">
+      <c r="O27" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O27" s="6" t="inlineStr">
+      <c r="P27" s="6" t="inlineStr">
         <is>
           <t>John D. Kaiser</t>
         </is>
       </c>
-      <c r="P27" s="6" t="inlineStr">
+      <c r="Q27" s="6" t="inlineStr">
         <is>
           <t>Murrieta CA</t>
         </is>
       </c>
-      <c r="Q27" s="6" t="inlineStr">
+      <c r="R27" s="6" t="inlineStr">
         <is>
           <t>Joseph J. Park</t>
         </is>
       </c>
-      <c r="R27" s="6" t="inlineStr">
+      <c r="S27" s="6" t="inlineStr">
         <is>
           <t>858-356-9070</t>
         </is>
       </c>
-      <c r="S27" s="11" t="inlineStr">
+      <c r="T27" s="11" t="inlineStr">
         <is>
           <t>25mo old; $350k+ equity; vacant/absentee; out-of-county heir</t>
         </is>
@@ -2604,59 +2939,60 @@
         </is>
       </c>
       <c r="B28" s="7" t="n"/>
-      <c r="C28" s="8" t="n"/>
+      <c r="C28" s="17" t="n"/>
       <c r="D28" s="7" t="n"/>
-      <c r="E28" s="8" t="n"/>
+      <c r="E28" s="17" t="n"/>
       <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
-      <c r="H28" s="9" t="n">
+      <c r="G28" s="18" t="n"/>
+      <c r="H28" s="7" t="n"/>
+      <c r="I28" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I28" s="10" t="n">
+      <c r="J28" s="19" t="n">
         <v>450000</v>
       </c>
-      <c r="J28" s="6" t="inlineStr">
+      <c r="K28" s="6" t="inlineStr">
         <is>
           <t>Albert Hanamey, aka Albert L. Hanamey</t>
         </is>
       </c>
-      <c r="K28" s="6" t="inlineStr">
+      <c r="L28" s="6" t="inlineStr">
         <is>
           <t>745 Pidgeon St.</t>
         </is>
       </c>
-      <c r="L28" s="6" t="inlineStr">
+      <c r="M28" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M28" s="6" t="n"/>
-      <c r="N28" s="6" t="inlineStr">
+      <c r="N28" s="6" t="n"/>
+      <c r="O28" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O28" s="6" t="inlineStr">
+      <c r="P28" s="6" t="inlineStr">
         <is>
           <t>Steven Albert-Hanamey Ferguson</t>
         </is>
       </c>
-      <c r="P28" s="6" t="inlineStr">
+      <c r="Q28" s="6" t="inlineStr">
         <is>
           <t>Seattle WA</t>
         </is>
       </c>
-      <c r="Q28" s="6" t="inlineStr">
+      <c r="R28" s="6" t="inlineStr">
         <is>
           <t>Pro Per</t>
         </is>
       </c>
-      <c r="R28" s="6" t="inlineStr">
+      <c r="S28" s="6" t="inlineStr">
         <is>
           <t>206-591-1650</t>
         </is>
       </c>
-      <c r="S28" s="11" t="inlineStr">
+      <c r="T28" s="11" t="inlineStr">
         <is>
           <t>27mo old; $350k+ equity; self-represented; out-of-county heir</t>
         </is>
@@ -2669,66 +3005,67 @@
         </is>
       </c>
       <c r="B29" s="7" t="n"/>
-      <c r="C29" s="8" t="n"/>
+      <c r="C29" s="17" t="n"/>
       <c r="D29" s="7" t="n"/>
-      <c r="E29" s="8" t="n"/>
+      <c r="E29" s="17" t="n"/>
       <c r="F29" s="7" t="n"/>
-      <c r="G29" s="7" t="n"/>
-      <c r="H29" s="9" t="n">
+      <c r="G29" s="18" t="n"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="I29" s="10" t="n">
+      <c r="J29" s="19" t="n">
         <v>380000</v>
       </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>Kenny Russell Johnson</t>
         </is>
       </c>
-      <c r="K29" s="6" t="inlineStr">
+      <c r="L29" s="6" t="inlineStr">
         <is>
           <t>2560 Street #20</t>
         </is>
       </c>
-      <c r="L29" s="6" t="inlineStr">
+      <c r="M29" s="6" t="inlineStr">
         <is>
           <t>San Diego</t>
         </is>
       </c>
-      <c r="M29" s="6" t="n"/>
-      <c r="N29" s="6" t="inlineStr">
+      <c r="N29" s="6" t="n"/>
+      <c r="O29" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="O29" s="6" t="inlineStr">
+      <c r="P29" s="6" t="inlineStr">
         <is>
           <t>Keith I. Johnson</t>
         </is>
       </c>
-      <c r="P29" s="6" t="inlineStr">
+      <c r="Q29" s="6" t="inlineStr">
         <is>
           <t>Fillmore CA</t>
         </is>
       </c>
-      <c r="Q29" s="6" t="inlineStr">
+      <c r="R29" s="6" t="inlineStr">
         <is>
           <t>Pro Per</t>
         </is>
       </c>
-      <c r="R29" s="6" t="inlineStr">
+      <c r="S29" s="6" t="inlineStr">
         <is>
           <t>626-483-5192 (*National DNC list)</t>
         </is>
       </c>
-      <c r="S29" s="11" t="inlineStr">
+      <c r="T29" s="11" t="inlineStr">
         <is>
           <t>27mo old; $350k+ equity; self-represented; out-of-county heir</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S29"/>
+  <autoFilter ref="A1:T29"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OPEN,CLOSED,DORMANT,NOT FOUND"</formula1>
@@ -2750,8 +3087,8 @@
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2761,12 +3098,15 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>11 of 28 A-tier cases verified against the court docket.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Fills in automatically as you work.</t>
-        </is>
-      </c>
+      <c r="A3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2793,97 +3133,88 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Dormant</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <f>COUNTIF(Verify!B2:B29,"DORMANT")</f>
+        <f>COUNTIF(Verify!B2:B29,"CLOSED")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Not yet checked</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF(Verify!B2:B29,"CLOSED")</f>
+        <f>28-B4</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="B8" s="3">
-        <f>COUNTIF(Verify!B2:B29,"NOT FOUND")</f>
-        <v/>
-      </c>
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Still live (open+dormant)</t>
-        </is>
-      </c>
-      <c r="B9" s="12">
-        <f>B5+B6</f>
+          <t>Open rate</t>
+        </is>
+      </c>
+      <c r="B9" s="13">
+        <f>IF(B4=0,"",B5/B4)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>% still live</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
-        <f>IF(B4=0,"",(B5+B6)/B4)</f>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Court-flagged delinquent</t>
+        </is>
+      </c>
+      <c r="B10" s="16">
+        <f>COUNTIF(Verify!G2:G29,"YES*")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Equity still live</t>
-        </is>
-      </c>
-      <c r="B11" s="14">
-        <f>SUMIFS(Verify!I2:I29,Verify!B2:B29,"OPEN")+SUMIFS(Verify!I2:I29,Verify!B2:B29,"DORMANT")</f>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Equity in open cases</t>
+        </is>
+      </c>
+      <c r="B11" s="31">
+        <f>SUMIF(Verify!B2:B29,"OPEN",Verify!J2:J29)</f>
         <v/>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Projected across all 423 aged cases</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Extrapolated to all 423 aged cases:</t>
-        </is>
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Est. still open</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>IF(B4=0,"",ROUND(B9*423,0))</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Est. still-live cases</t>
-        </is>
-      </c>
-      <c r="B15" s="3">
-        <f>IF(B4=0,"",ROUND(B10*423,0))</f>
-        <v/>
-      </c>
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>…as % of your pipeline</t>
-        </is>
-      </c>
-      <c r="B16" s="16">
-        <f>IF(B4=0,"",B10)</f>
-        <v/>
-      </c>
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="16" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Complete A-tier verification: 10 of 28 still open
Marks the remaining 17 cases closed per docket check. Final A-tier open
rate is 36%, well below the 91% the first 11 suggested.

Records that the priority score has no predictive power for open vs
closed status (open mean 53.0, closed mean 53.3), so ranking and status
verification must be treated as independent steps.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KmrMHojnrvSNV7tKWJ6vCj
</commit_message>
<xml_diff>
--- a/San_Diego_ATier_Verification_Tracker.xlsx
+++ b/San_Diego_ATier_Verification_Tracker.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +79,11 @@
     <font>
       <b val="1"/>
       <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -141,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -182,6 +187,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -886,13 +892,29 @@
           <t>24PE001139C</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n"/>
-      <c r="C2" s="17" t="n"/>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="17" t="n"/>
-      <c r="F2" s="7" t="n"/>
-      <c r="G2" s="18" t="n"/>
-      <c r="H2" s="7" t="n"/>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C2" s="27" t="n"/>
+      <c r="D2" s="28" t="n"/>
+      <c r="E2" s="27" t="n"/>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G2" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H2" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I2" s="9" t="n">
         <v>73</v>
       </c>
@@ -956,13 +978,29 @@
           <t>24PE000313C</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n"/>
-      <c r="C3" s="17" t="n"/>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="17" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="18" t="n"/>
-      <c r="H3" s="7" t="n"/>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="28" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G3" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H3" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I3" s="9" t="n">
         <v>66</v>
       </c>
@@ -1026,13 +1064,29 @@
           <t>24PE001223C</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="17" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="17" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="18" t="n"/>
-      <c r="H4" s="7" t="n"/>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="28" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H4" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I4" s="9" t="n">
         <v>61</v>
       </c>
@@ -1190,13 +1244,29 @@
           <t>24PE001244C</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="18" t="n"/>
-      <c r="H6" s="7" t="n"/>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="28" t="n"/>
+      <c r="E6" s="27" t="n"/>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H6" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I6" s="9" t="n">
         <v>60</v>
       </c>
@@ -1260,13 +1330,29 @@
           <t>24PE001359C</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="7" t="n"/>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="28" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H7" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I7" s="9" t="n">
         <v>60</v>
       </c>
@@ -1612,13 +1698,29 @@
           <t>24PE001404C</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="18" t="n"/>
-      <c r="H11" s="7" t="n"/>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="n"/>
+      <c r="D11" s="28" t="n"/>
+      <c r="E11" s="27" t="n"/>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G11" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I11" s="9" t="n">
         <v>54</v>
       </c>
@@ -1678,13 +1780,29 @@
           <t>24PE000304C</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="18" t="n"/>
-      <c r="H12" s="7" t="n"/>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="n"/>
+      <c r="D12" s="28" t="n"/>
+      <c r="E12" s="27" t="n"/>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H12" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I12" s="9" t="n">
         <v>54</v>
       </c>
@@ -2018,13 +2136,29 @@
           <t>24PE000351C</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="17" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="7" t="n"/>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="n"/>
+      <c r="D16" s="28" t="n"/>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H16" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I16" s="9" t="n">
         <v>51</v>
       </c>
@@ -2180,13 +2314,29 @@
           <t>24PE000969C</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="17" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="7" t="n"/>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="n"/>
+      <c r="D18" s="28" t="n"/>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G18" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H18" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I18" s="9" t="n">
         <v>50</v>
       </c>
@@ -2344,13 +2494,29 @@
           <t>24PE001484C</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="17" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="17" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="18" t="n"/>
-      <c r="H20" s="7" t="n"/>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="n"/>
+      <c r="D20" s="28" t="n"/>
+      <c r="E20" s="27" t="n"/>
+      <c r="F20" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G20" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H20" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I20" s="9" t="n">
         <v>48</v>
       </c>
@@ -2414,13 +2580,29 @@
           <t>24PE001502C</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="17" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="18" t="n"/>
-      <c r="H21" s="7" t="n"/>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="n"/>
+      <c r="D21" s="28" t="n"/>
+      <c r="E21" s="27" t="n"/>
+      <c r="F21" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G21" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H21" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I21" s="9" t="n">
         <v>47</v>
       </c>
@@ -2574,13 +2756,29 @@
           <t>24PE000986C</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="17" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="7" t="n"/>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="n"/>
+      <c r="D23" s="28" t="n"/>
+      <c r="E23" s="27" t="n"/>
+      <c r="F23" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G23" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H23" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I23" s="9" t="n">
         <v>47</v>
       </c>
@@ -2736,13 +2934,29 @@
           <t>24PE001085C</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="17" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="7" t="n"/>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C25" s="27" t="n"/>
+      <c r="D25" s="28" t="n"/>
+      <c r="E25" s="27" t="n"/>
+      <c r="F25" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G25" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H25" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I25" s="9" t="n">
         <v>47</v>
       </c>
@@ -2802,13 +3016,29 @@
           <t>24PE001042C</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="17" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="17" t="n"/>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="7" t="n"/>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C26" s="27" t="n"/>
+      <c r="D26" s="28" t="n"/>
+      <c r="E26" s="27" t="n"/>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G26" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H26" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I26" s="9" t="n">
         <v>47</v>
       </c>
@@ -2868,13 +3098,29 @@
           <t>24PE001528C</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="17" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="17" t="n"/>
-      <c r="F27" s="7" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="7" t="n"/>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="n"/>
+      <c r="D27" s="28" t="n"/>
+      <c r="E27" s="27" t="n"/>
+      <c r="F27" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G27" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H27" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I27" s="9" t="n">
         <v>47</v>
       </c>
@@ -2938,13 +3184,29 @@
           <t>24PE000983C</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="17" t="n"/>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="17" t="n"/>
-      <c r="F28" s="7" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="7" t="n"/>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="28" t="n"/>
+      <c r="E28" s="27" t="n"/>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G28" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H28" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I28" s="9" t="n">
         <v>47</v>
       </c>
@@ -3004,13 +3266,29 @@
           <t>24PE000854C</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="17" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="17" t="n"/>
-      <c r="F29" s="7" t="n"/>
-      <c r="G29" s="18" t="n"/>
-      <c r="H29" s="7" t="n"/>
+      <c r="B29" s="26" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="n"/>
+      <c r="D29" s="28" t="n"/>
+      <c r="E29" s="27" t="n"/>
+      <c r="F29" s="28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G29" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H29" s="30" t="inlineStr">
+        <is>
+          <t>Closed - confirmed by Palmer from the court docket. Not parsed from a ROA PDF in this session, so no last-activity or discharge date recorded.</t>
+        </is>
+      </c>
       <c r="I29" s="9" t="n">
         <v>47</v>
       </c>
@@ -3084,24 +3362,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Results</t>
+          <t>Results - A-Tier Verification Complete</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>11 of 28 A-tier cases verified against the court docket.</t>
+          <t>All 28 A-tier cases checked against the court docket.</t>
         </is>
       </c>
     </row>
@@ -3122,7 +3400,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Still open</t>
         </is>
       </c>
       <c r="B5" s="3">
@@ -3142,70 +3420,74 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Not yet checked</t>
-        </is>
-      </c>
-      <c r="B7" s="3">
-        <f>28-B4</f>
-        <v/>
-      </c>
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Open rate</t>
         </is>
       </c>
-      <c r="B9" s="13">
+      <c r="B8" s="13">
         <f>IF(B4=0,"",B5/B4)</f>
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Court-flagged delinquent</t>
+        </is>
+      </c>
+      <c r="B9" s="16">
+        <f>COUNTIF(Verify!G2:G29,"YES*")</f>
+        <v/>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Court-flagged delinquent</t>
-        </is>
-      </c>
-      <c r="B10" s="16">
-        <f>COUNTIF(Verify!G2:G29,"YES*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
           <t>Equity in open cases</t>
         </is>
       </c>
-      <c r="B11" s="31">
+      <c r="B10" s="31">
         <f>SUMIF(Verify!B2:B29,"OPEN",Verify!J2:J29)</f>
         <v/>
       </c>
     </row>
-    <row r="12"/>
+    <row r="11">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="31" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Projected across all 423 aged cases</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Projected across all 423 aged cases</t>
-        </is>
+          <t>Est. still open (point estimate)</t>
+        </is>
+      </c>
+      <c r="B13" s="12">
+        <f>ROUND(B8*423,0)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Est. still open</t>
-        </is>
-      </c>
-      <c r="B14" s="12">
-        <f>IF(B4=0,"",ROUND(B9*423,0))</f>
-        <v/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Plausible range (95% CI)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>76 to 226</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -3213,8 +3495,26 @@
       <c r="B15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
+      <c r="A16" s="32" t="inlineStr">
+        <is>
+          <t>Note: the priority score does not predict open vs closed.</t>
+        </is>
+      </c>
       <c r="B16" s="16" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Open cases averaged 53.0, closed averaged 53.3. Rank by score for deal value;</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>check the docket separately for status. The two are independent.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>